<commit_message>
Update TTK equipment options and templates.
Add the Sony FE 70-200 lens to both TTK modes, place it between FX3 and Panasonic in the form/export, and allow selecting it only when FX3 is chosen.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/excel_templates/ttk_without_main_kit_template.xlsx
+++ b/excel_templates/ttk_without_main_kit_template.xlsx
@@ -1325,7 +1325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="75" customWidth="1" min="1" max="1"/>
@@ -1761,46 +1761,64 @@
       </c>
       <c r="D29" s="62" t="n"/>
     </row>
-    <row r="30" ht="46" customHeight="1" thickBot="1">
+    <row r="30" ht="22" customHeight="1" thickBot="1">
       <c r="A30" s="53" t="n"/>
       <c r="B30" s="57" t="inlineStr">
         <is>
+          <t>Объектив Sony FE 2.8 /70-200 GM OSS</t>
+        </is>
+      </c>
+      <c r="C30" s="52" t="inlineStr">
+        <is>
+          <t>???</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="n"/>
+    </row>
+    <row r="31" ht="22" customHeight="1" thickBot="1">
+      <c r="A31" s="53" t="n"/>
+      <c r="B31" s="57" t="inlineStr">
+        <is>
           <t>Камера Panasonic AJ-PX270</t>
         </is>
       </c>
-      <c r="C30" s="52" t="inlineStr">
+      <c r="C31" s="52" t="inlineStr">
         <is>
           <t>???</t>
         </is>
       </c>
-      <c r="D30" s="14" t="n"/>
-    </row>
-    <row r="31" ht="22" customHeight="1" thickBot="1">
-      <c r="A31" s="22" t="inlineStr">
+      <c r="D31" s="14" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="22" t="inlineStr">
         <is>
           <t>Дата и  Время сдачи материала в  инжест</t>
         </is>
       </c>
-      <c r="B31" s="55" t="inlineStr">
+      <c r="B32" s="55" t="inlineStr">
         <is>
           <t xml:space="preserve">Инженер инжеста ФИО </t>
         </is>
       </c>
-      <c r="C31" s="51" t="inlineStr">
+      <c r="C32" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">Подпись </t>
         </is>
       </c>
-      <c r="D31" s="23" t="n"/>
-    </row>
-    <row r="36" ht="41.25" customHeight="1">
-      <c r="B36" s="2" t="n"/>
-    </row>
+      <c r="D32" s="23" t="n"/>
+    </row>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36" ht="41.25" customHeight="1"/>
     <row r="37" ht="19" customHeight="1">
       <c r="B37" s="2" t="n"/>
     </row>
     <row r="38" ht="69.75" customHeight="1">
       <c r="B38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>